<commit_message>
Update Schedule.xlsx after scheduled run
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -2111,7 +2111,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Pending (sends 16/09/2026, 5 day(s) before Date 21/09/2026)</t>
+          <t>Sent (16/09/2026)</t>
         </is>
       </c>
       <c r="K30" s="17">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Pending (sends 16/09/2026, 5 day(s) before Date 21/09/2026)</t>
+          <t>Sent (16/09/2026)</t>
         </is>
       </c>
       <c r="K48" s="17">

</xml_diff>

<commit_message>
Support yearly-recurring Date spec; add Surat quarterly PT rows
"N Every month" was the only recognized recurring pattern -- a row like
"15 July every Year" matched neither that nor a literal date, so it
would have been marked Error: bad/missing Date and never sent. Added
parse_recurring_yearly()/this_years_occurrence() to resolve "DD Month
every Year" specs the same way monthly ones already work.

Also fixed a stray leading space in the rendered message when {label}
is empty, and added the 4 new Surat quarterly professional-tax rows.
The 3 deadlines that already passed this year (Jan/Apr/Jul) are marked
Skipped so they don't fire a stale notice; they resume normally next
year. The upcoming Oct row is untouched and will send 5 days before,
as usual.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Emails" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="[$-409]dd/mmm/yy;@"/>
     <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="167" formatCode="dd\/mm\/yyyy"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -33,12 +33,14 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
@@ -143,7 +145,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,6 +194,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,10 +570,10 @@
   <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" style="21" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1">
+    <row r="1" ht="17" customHeight="1" s="21">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Scheduled Mass Mail -- how this workbook works</t>
@@ -767,18 +773,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="31.1796875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="110.26953125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" style="21" min="1" max="1"/>
+    <col width="26" customWidth="1" style="21" min="2" max="2"/>
+    <col width="22" customWidth="1" style="21" min="4" max="4"/>
+    <col width="42" customWidth="1" style="21" min="6" max="6"/>
+    <col width="14.1796875" bestFit="1" customWidth="1" style="21" min="7" max="7"/>
+    <col width="31.1796875" bestFit="1" customWidth="1" style="21" min="8" max="8"/>
+    <col width="110.26953125" bestFit="1" customWidth="1" style="21" min="9" max="9"/>
+    <col width="22" customWidth="1" style="21" min="10" max="10"/>
+    <col width="12" customWidth="1" style="21" min="11" max="11"/>
+    <col width="17.1796875" bestFit="1" customWidth="1" style="21" min="12" max="12"/>
+    <col width="10.54296875" bestFit="1" customWidth="1" style="21" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -853,7 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="101.5" customHeight="1" s="21">
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>hr@indigopaints.com</t>
@@ -867,10 +875,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I2" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -897,7 +906,7 @@
         <v>46548</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="101.5" customHeight="1" s="21">
       <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Ranchi@indigopaints.com</t>
@@ -911,10 +920,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -941,7 +951,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="101.5" customHeight="1" s="21">
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Patna@indigopaints.com</t>
@@ -955,10 +965,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -985,7 +996,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="101.5" customHeight="1" s="21">
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>kochi@indigopaints.com</t>
@@ -999,10 +1010,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1029,7 +1041,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="101.5" customHeight="1" s="21">
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>kochi@indigopaints.com</t>
@@ -1043,10 +1055,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1073,7 +1086,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="101.5" customHeight="1" s="21">
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Calicut@indigopaints.com</t>
@@ -1087,10 +1100,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1117,7 +1131,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="101.5" customHeight="1" s="21">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Calicut@indigopaints.com</t>
@@ -1131,10 +1145,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1161,7 +1176,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="101.5" customHeight="1" s="21">
       <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Kollam@indigopaints.com</t>
@@ -1175,10 +1190,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1205,7 +1221,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="101.5" customHeight="1" s="21">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Kollam@indigopaints.com</t>
@@ -1219,10 +1235,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1249,7 +1266,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="101.5" customHeight="1" s="21">
       <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Thrissur@indigopaints.com</t>
@@ -1263,10 +1280,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1293,7 +1311,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="101.5" customHeight="1" s="21">
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Thrissur@indigopaints.com</t>
@@ -1307,10 +1325,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1337,7 +1356,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="101.5" customHeight="1" s="21">
       <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Indore@indigopaints.com</t>
@@ -1351,10 +1370,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1381,7 +1401,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="101.5" customHeight="1" s="21">
       <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Kolkata@indigopaints.com</t>
@@ -1395,10 +1415,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1425,7 +1446,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="101.5" customHeight="1" s="21">
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Cuttack@indigopaints.com</t>
@@ -1439,10 +1460,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1469,7 +1491,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="101.5" customHeight="1" s="21">
       <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Vizag@indigopaints.com , Vijayawada@indigopaints.com</t>
@@ -1483,10 +1505,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1513,7 +1536,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="101.5" customHeight="1" s="21">
       <c r="B17" s="4" t="inlineStr">
         <is>
           <t>ahmedabad@indigopaints.com</t>
@@ -1527,10 +1550,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I17" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1557,7 +1581,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="101.5" customHeight="1" s="21">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Surat@indigopaints.com</t>
@@ -1571,10 +1595,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1601,7 +1626,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="101.5" customHeight="1" s="21">
       <c r="B19" s="4" t="inlineStr">
         <is>
           <t>rajkot@indigopaints.com</t>
@@ -1615,10 +1640,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1645,7 +1671,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="101.5" customHeight="1" s="21">
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>guwahati@indigopaints.com</t>
@@ -1659,10 +1685,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I20" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1689,7 +1716,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="101.5" customHeight="1" s="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Chennai@indigopaints.com</t>
@@ -1703,10 +1730,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I21" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1733,7 +1761,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="101.5" customHeight="1" s="21">
       <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Chennai@indigopaints.com</t>
@@ -1747,10 +1775,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I22" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1777,7 +1806,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="101.5" customHeight="1" s="21">
       <c r="B23" s="4" t="inlineStr">
         <is>
           <t>madurai@indigopaints.com</t>
@@ -1791,10 +1820,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I23" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1821,7 +1851,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="101.5" customHeight="1" s="21">
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>madurai@indigopaints.com</t>
@@ -1835,10 +1865,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I24" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1865,7 +1896,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="101.5" customHeight="1" s="21">
       <c r="B25" s="4" t="inlineStr">
         <is>
           <t>coimbatore@indigopaints.com</t>
@@ -1879,10 +1910,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I25" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1909,7 +1941,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="101.5" customHeight="1" s="21">
       <c r="B26" s="4" t="inlineStr">
         <is>
           <t>coimbatore@indigopaints.com</t>
@@ -1923,10 +1955,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1953,7 +1986,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="101.5" customHeight="1" s="21">
       <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Bengaluru@indigopaints.com , hubli@indigopaints.com</t>
@@ -1967,10 +2000,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I27" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -1997,7 +2031,7 @@
         <v>46137</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="101.5" customHeight="1" s="21">
       <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Hyderabad@indigopaints.com</t>
@@ -2011,10 +2045,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I28" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2041,7 +2076,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="101.5" customHeight="1" s="21">
       <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Ludhiana@indigopaints.com , jalandhar@indigopaints.com , zirakpur@indigopaints.com</t>
@@ -2055,10 +2090,11 @@
           <t xml:space="preserve">Employer professional tax due date </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I29" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2085,7 +2121,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="101.5" customHeight="1" s="21">
       <c r="B30" s="3" t="inlineStr">
         <is>
           <t>hr@indigopaints.com</t>
@@ -2101,10 +2137,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I30" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2131,7 +2168,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="101.5" customHeight="1" s="21">
       <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Ranchi@indigopaints.com</t>
@@ -2147,10 +2184,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I31" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2177,7 +2215,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="101.5" customHeight="1" s="21">
       <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Patna@indigopaints.com</t>
@@ -2193,10 +2231,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I32" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2223,7 +2262,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="101.5" customHeight="1" s="21">
       <c r="B33" s="3" t="inlineStr">
         <is>
           <t>pdktaccounts@indigopaints.com</t>
@@ -2237,10 +2276,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I33" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2267,7 +2307,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="101.5" customHeight="1" s="21">
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>pdktaccounts@indigopaints.com</t>
@@ -2281,10 +2321,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I34" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2311,7 +2352,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="101.5" customHeight="1" s="21">
       <c r="B35" s="5" t="inlineStr">
         <is>
           <t>kochi@indigopaints.com</t>
@@ -2325,10 +2366,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I35" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2355,7 +2397,7 @@
         <v>46260</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="101.5" customHeight="1" s="21">
       <c r="B36" s="5" t="inlineStr">
         <is>
           <t>kochi@indigopaints.com</t>
@@ -2369,10 +2411,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I36" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2399,7 +2442,7 @@
         <v>46441</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="101.5" customHeight="1" s="21">
       <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Kollam@indigopaints.com</t>
@@ -2413,10 +2456,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I37" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2443,7 +2487,7 @@
         <v>46260</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="101.5" customHeight="1" s="21">
       <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Kollam@indigopaints.com</t>
@@ -2457,10 +2501,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I38" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2487,7 +2532,7 @@
         <v>46441</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="101.5" customHeight="1" s="21">
       <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Thrissur@indigopaints.com</t>
@@ -2501,10 +2546,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I39" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2531,7 +2577,7 @@
         <v>46260</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="101.5" customHeight="1" s="21">
       <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Thrissur@indigopaints.com</t>
@@ -2545,10 +2591,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I40" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2575,7 +2622,7 @@
         <v>46441</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="101.5" customHeight="1" s="21">
       <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Indore@indigopaints.com</t>
@@ -2591,10 +2638,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I41" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2621,7 +2669,7 @@
         <v>46270</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="101.5" customHeight="1" s="21">
       <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Kolkata@indigopaints.com</t>
@@ -2637,10 +2685,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I42" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2667,7 +2716,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="101.5" customHeight="1" s="21">
       <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Cuttack@indigopaints.com</t>
@@ -2683,10 +2732,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I43" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2713,7 +2763,7 @@
         <v>46270</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="101.5" customHeight="1" s="21">
       <c r="B44" s="7" t="inlineStr">
         <is>
           <t>Vizag@indigopaints.com , Vijayawada@indigopaints.com</t>
@@ -2729,10 +2779,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I44" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2759,7 +2810,7 @@
         <v>46270</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="101.5" customHeight="1" s="21">
       <c r="B45" s="4" t="inlineStr">
         <is>
           <t>ahmedabad@indigopaints.com</t>
@@ -2775,10 +2826,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I45" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2805,7 +2857,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="101.5" customHeight="1" s="21">
       <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Surat@indigopaints.com</t>
@@ -2821,10 +2873,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I46" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2851,7 +2904,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="101.5" customHeight="1" s="21">
       <c r="B47" s="4" t="inlineStr">
         <is>
           <t>rajkot@indigopaints.com</t>
@@ -2867,10 +2920,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I47" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2897,7 +2951,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="101.5" customHeight="1" s="21">
       <c r="B48" s="4" t="inlineStr">
         <is>
           <t>guwahati@indigopaints.com</t>
@@ -2913,10 +2967,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I48" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2943,7 +2998,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="101.5" customHeight="1" s="21">
       <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Chennai@indigopaints.com</t>
@@ -2957,10 +3012,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I49" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -2987,7 +3043,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="101.5" customHeight="1" s="21">
       <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Chennai@indigopaints.com</t>
@@ -3001,10 +3057,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I50" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3031,7 +3088,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="101.5" customHeight="1" s="21">
       <c r="B51" s="4" t="inlineStr">
         <is>
           <t>madurai@indigopaints.com</t>
@@ -3045,10 +3102,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I51" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3075,7 +3133,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="101.5" customHeight="1" s="21">
       <c r="B52" s="4" t="inlineStr">
         <is>
           <t>madurai@indigopaints.com</t>
@@ -3089,10 +3147,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I52" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3119,7 +3178,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="101.5" customHeight="1" s="21">
       <c r="B53" s="4" t="inlineStr">
         <is>
           <t>coimbatore@indigopaints.com</t>
@@ -3133,10 +3192,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I53" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3163,7 +3223,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="101.5" customHeight="1" s="21">
       <c r="B54" s="4" t="inlineStr">
         <is>
           <t>coimbatore@indigopaints.com</t>
@@ -3177,10 +3237,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I54" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3207,7 +3268,7 @@
         <v>46472</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="101.5" customHeight="1" s="21">
       <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Bengaluru@indigopaints.com , hubli@indigopaints.com</t>
@@ -3223,10 +3284,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I55" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3253,7 +3315,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="101.5" customHeight="1" s="21">
       <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Hyderabad@indigopaints.com</t>
@@ -3269,10 +3331,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I56" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3299,7 +3362,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="101.5" customHeight="1" s="21">
       <c r="B57" s="4" t="inlineStr">
         <is>
           <t>Ludhiana@indigopaints.com</t>
@@ -3315,10 +3378,11 @@
           <t xml:space="preserve">Employee professional tax due date </t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I57" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3345,7 +3409,7 @@
         <v>46286</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="101.5" customHeight="1" s="21">
       <c r="B58" s="6" t="inlineStr">
         <is>
           <t>jodhpur@indigopaints.com</t>
@@ -3361,10 +3425,11 @@
           <t>ESIC</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I58" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3391,7 +3456,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="101.5" customHeight="1" s="21">
       <c r="B59" s="5" t="inlineStr">
         <is>
           <t>kochi@indigopaints.com</t>
@@ -3407,10 +3472,11 @@
           <t>ESIC</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I59" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3437,7 +3503,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="101.5" customHeight="1" s="21">
       <c r="B60" s="5" t="inlineStr">
         <is>
           <t>pdktaccounts@indigopaints.com</t>
@@ -3453,10 +3519,11 @@
           <t>ESIC</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I60" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3483,7 +3550,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="101.5" customHeight="1" s="21">
       <c r="B61" s="6" t="inlineStr">
         <is>
           <t>jodhpur@indigopaints.com</t>
@@ -3499,10 +3566,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I61" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3529,7 +3597,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="101.5" customHeight="1" s="21">
       <c r="B62" s="3" t="inlineStr">
         <is>
           <t>somnath@indigopaints.com</t>
@@ -3545,10 +3613,11 @@
           <t>TDS</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+      <c r="I62" s="20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
@@ -3573,6 +3642,133 @@
       </c>
       <c r="N62" s="19" t="n">
         <v>46267</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> surat@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>15 July every Year</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>PT due date is quarterly.</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Skipped (10/07/2026)</t>
+        </is>
+      </c>
+      <c r="K63" s="17">
+        <f>IFERROR(IF(ISNUMBER($G63),DAY($G63),VALUE(LEFT(TRIM($G63),FIND(" ",TRIM($G63))-1))),"")</f>
+        <v/>
+      </c>
+      <c r="L63" s="18">
+        <f>IF(ISNUMBER($G63),$G63,IF(DAY(TODAY())&lt;=$K63,DATE(YEAR(TODAY()),MONTH(TODAY()),MIN($K63,DAY(EOMONTH(TODAY(),0)))),DATE(YEAR(TODAY()),MONTH(TODAY())+1,MIN($K63,DAY(EOMONTH(TODAY(),1))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> surat@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>15 October every Year</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>PT due date is quarterly.</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> surat@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>15 January every Year</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>PT due date is quarterly.</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Skipped (10/01/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> surat@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>15 April every Year</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>PT due date is quarterly.</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;{label} due date - {date} &lt;/p&gt;
+&lt;p&gt;Note: If the due date falls on a Sunday or public holiday, please ensure that the payment is made before the Sunday or holiday to avoid any delay or penalty.&lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Skipped (10/04/2026)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3584,8 +3780,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" display="kochi@indigopaints.com" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" display="kochi@indigopaints.com" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" display="Vizag@indigopaints.com , " r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId12"/>

</xml_diff>